<commit_message>
RF05b: integra matching, reservas e recuperação por Kafka
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/risco.xlsx
+++ b/frontend/runner/exemplos/risco.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="115">
   <si>
     <t>cenario</t>
   </si>
@@ -66,7 +66,7 @@
     <t>{"content-type":"application/json"}</t>
   </si>
   <si>
-    <t>{"saldo":"100.00","custodia":{}}</t>
+    <t>{"saldo":"100.00","custodia":{"ALFA3":7}}</t>
   </si>
   <si>
     <t/>
@@ -75,7 +75,7 @@
     <t>ReservaCustodia</t>
   </si>
   <si>
-    <t>{"saldo":"0.00","custodia":{"GAMA3":5}}</t>
+    <t>{"saldo":"150.00","custodia":{"GAMA3":5}}</t>
   </si>
   <si>
     <t>MarketTeto</t>
@@ -84,18 +84,21 @@
     <t>{"saldo":"219.99","custodia":{}}</t>
   </si>
   <si>
+    <t>QuantidadeMaxima</t>
+  </si>
+  <si>
+    <t>{"saldo":"2000000.00","custodia":{"ALFA3":100000}}</t>
+  </si>
+  <si>
     <t>OcoReservaUnica</t>
   </si>
   <si>
+    <t>/api/v1/preparacoes-risco/contas/CONTA-003</t>
+  </si>
+  <si>
     <t>{"saldo":"1000.00","custodia":{}}</t>
   </si>
   <si>
-    <t>QuantidadeMaxima</t>
-  </si>
-  <si>
-    <t>{"saldo":"2000000.00","custodia":{}}</t>
-  </si>
-  <si>
     <t>Primeira</t>
   </si>
   <si>
@@ -153,6 +156,27 @@
     <t>Inalterado</t>
   </si>
   <si>
+    <t>Contraparte</t>
+  </si>
+  <si>
+    <t>{"content-type":"application/json","x-idempotency-key":"${cenario}-3"}</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"IOC","quantidade":7,"precoLimite":"10.00"}</t>
+  </si>
+  <si>
+    <t>{"limpeza":"/id"}</t>
+  </si>
+  <si>
+    <t>Executada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${limpeza}</t>
+  </si>
+  <si>
+    <t>Liberado</t>
+  </si>
+  <si>
     <t>Excedente</t>
   </si>
   <si>
@@ -174,6 +198,9 @@
     <t>CustodiaReservada</t>
   </si>
   <si>
+    <t>{"ticker":"GAMA3","lado":"COMPRA","tipo":"LIMIT","validade":"IOC","quantidade":5,"precoLimite":"30.00"}</t>
+  </si>
+  <si>
     <t>Insuficiente</t>
   </si>
   <si>
@@ -195,12 +222,54 @@
     <t>SuficienteReservada</t>
   </si>
   <si>
-    <t>TetoReservado</t>
+    <t>TetoLiberado</t>
+  </si>
+  <si>
+    <t>Acima</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100001,"precoLimite":"10.00"}</t>
+  </si>
+  <si>
+    <t>AcimaRejeitada</t>
+  </si>
+  <si>
+    <t>NoLimite</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100000,"precoLimite":"10.00"}</t>
+  </si>
+  <si>
+    <t>NoLimiteReservada</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"IOC","quantidade":100000,"precoLimite":"10.00"}</t>
+  </si>
+  <si>
+    <t>Isolamento</t>
+  </si>
+  <si>
+    <t>OutraConta</t>
+  </si>
+  <si>
+    <t>risco-b</t>
+  </si>
+  <si>
+    <t>ContaDaTela</t>
+  </si>
+  <si>
+    <t>/api/v1/preparacoes-risco/contas/CONTA-001</t>
+  </si>
+  <si>
+    <t>{"saldo":"1.00"}</t>
   </si>
   <si>
     <t>Enviar</t>
   </si>
   <si>
+    <t>ordens-b</t>
+  </si>
+  <si>
     <t>/api/v1/ordens-oco</t>
   </si>
   <si>
@@ -219,42 +288,6 @@
     <t>ReservaUnica</t>
   </si>
   <si>
-    <t>Acima</t>
-  </si>
-  <si>
-    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100001,"precoLimite":"10.00"}</t>
-  </si>
-  <si>
-    <t>AcimaRejeitada</t>
-  </si>
-  <si>
-    <t>NoLimite</t>
-  </si>
-  <si>
-    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100000,"precoLimite":"10.00"}</t>
-  </si>
-  <si>
-    <t>NoLimiteReservada</t>
-  </si>
-  <si>
-    <t>Isolamento</t>
-  </si>
-  <si>
-    <t>OutraConta</t>
-  </si>
-  <si>
-    <t>risco-b</t>
-  </si>
-  <si>
-    <t>ContaDaTela</t>
-  </si>
-  <si>
-    <t>/api/v1/preparacoes-risco/contas/CONTA-001</t>
-  </si>
-  <si>
-    <t>{"saldo":"1.00"}</t>
-  </si>
-  <si>
     <t>passo</t>
   </si>
   <si>
@@ -270,7 +303,7 @@
     <t>{"/estado":"RECEBIDA"}</t>
   </si>
   <si>
-    <t>{"/estado":"RESERVADA","/motivoRejeicao":null}</t>
+    <t>{"/estado":"ABERTA","/motivoRejeicao":null}</t>
   </si>
   <si>
     <t>{"/saldoDisponivel":"30.00","/saldoReservado":"70.00"}</t>
@@ -279,16 +312,43 @@
     <t>{"/estado":"REJEITADA","/motivoRejeicao":"SALDO_INSUFICIENTE"}</t>
   </si>
   <si>
+    <t>{"/estado":"EXECUTADA","/motivoRejeicao":null}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"30.00","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
     <t>{"/estado":"REJEITADA","/motivoRejeicao":"CUSTODIA_INSUFICIENTE"}</t>
   </si>
   <si>
     <t>{"/custodias/3/ticker":"GAMA3","/custodias/3/disponivel":0,"/custodias/3/reservado":5}</t>
   </si>
   <si>
+    <t>{"/saldoTotal":"0.00","/saldoReservado":"0.00","/custodias/3/reservado":0}</t>
+  </si>
+  <si>
     <t>{"/saldoDisponivel":"220.00"}</t>
   </si>
   <si>
-    <t>{"/saldoDisponivel":"0.00","/saldoReservado":"220.00"}</t>
+    <t>{"/estado":"CANCELADA","/motivoRejeicao":null}</t>
+  </si>
+  <si>
+    <t>{"/saldoDisponivel":"220.00","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
+    <t>{"/estado":"REJEITADA","/motivoRejeicao":"QUANTIDADE_MAXIMA_EXCEDIDA"}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"1000000.00","/saldoReservado":"0.00"}</t>
+  </si>
+  <si>
+    <t>{"/conta":"CONTA-003"}</t>
+  </si>
+  <si>
+    <t>{"/codigo":"CONTA_NAO_PREPARAVEL"}</t>
+  </si>
+  <si>
+    <t>{"/conta":"CONTA-003","/saldoReservado":"0.00"}</t>
   </si>
   <si>
     <t>{}</t>
@@ -298,15 +358,6 @@
   </si>
   <si>
     <t>{"/saldoDisponivel":"769.00","/saldoReservado":"231.00"}</t>
-  </si>
-  <si>
-    <t>{"/estado":"REJEITADA","/motivoRejeicao":"QUANTIDADE_MAXIMA_EXCEDIDA"}</t>
-  </si>
-  <si>
-    <t>{"/conta":"CONTA-003"}</t>
-  </si>
-  <si>
-    <t>{"/codigo":"CONTA_NAO_PREPARAVEL"}</t>
   </si>
 </sst>
 </file>
@@ -878,13 +929,13 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
         <v>16</v>
       </c>
       <c r="H6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
@@ -904,7 +955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -950,25 +1001,25 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
         <v>18</v>
@@ -985,16 +1036,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
         <v>18</v>
@@ -1020,16 +1071,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" t="s">
         <v>18</v>
@@ -1040,11 +1091,11 @@
       <c r="I4" t="s">
         <v>18</v>
       </c>
-      <c r="J4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" t="s">
-        <v>18</v>
+      <c r="J4">
+        <v>200</v>
+      </c>
+      <c r="K4">
+        <v>15000</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1055,25 +1106,25 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J5" t="s">
         <v>18</v>
@@ -1090,16 +1141,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
         <v>18</v>
@@ -1125,16 +1176,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
         <v>18</v>
@@ -1145,40 +1196,40 @@
       <c r="I7" t="s">
         <v>18</v>
       </c>
-      <c r="J7" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" t="s">
-        <v>18</v>
+      <c r="J7">
+        <v>200</v>
+      </c>
+      <c r="K7">
+        <v>15000</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I8" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="J8" t="s">
         <v>18</v>
@@ -1189,22 +1240,22 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
@@ -1224,37 +1275,37 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="H10" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="I10" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="J10">
+        <v>200</v>
+      </c>
+      <c r="K10">
+        <v>15000</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1262,34 +1313,34 @@
         <v>19</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H11" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="I11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11">
-        <v>200</v>
-      </c>
-      <c r="K11">
-        <v>15000</v>
+        <v>34</v>
+      </c>
+      <c r="J11" t="s">
+        <v>18</v>
+      </c>
+      <c r="K11" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1297,19 +1348,19 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G12" t="s">
         <v>18</v>
@@ -1320,40 +1371,40 @@
       <c r="I12" t="s">
         <v>18</v>
       </c>
-      <c r="J12" t="s">
-        <v>18</v>
-      </c>
-      <c r="K12" t="s">
-        <v>18</v>
+      <c r="J12">
+        <v>200</v>
+      </c>
+      <c r="K12">
+        <v>15000</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="H13" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I13" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="J13" t="s">
         <v>18</v>
@@ -1364,22 +1415,22 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G14" t="s">
         <v>18</v>
@@ -1399,66 +1450,66 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H15" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="I15" t="s">
         <v>18</v>
       </c>
-      <c r="J15" t="s">
-        <v>18</v>
-      </c>
-      <c r="K15" t="s">
-        <v>18</v>
+      <c r="J15">
+        <v>200</v>
+      </c>
+      <c r="K15">
+        <v>15000</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G16" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="H16" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I16" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="J16" t="s">
         <v>18</v>
@@ -1469,22 +1520,22 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G17" t="s">
         <v>18</v>
@@ -1504,22 +1555,22 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G18" t="s">
         <v>18</v>
@@ -1530,40 +1581,40 @@
       <c r="I18" t="s">
         <v>18</v>
       </c>
-      <c r="J18" t="s">
-        <v>18</v>
-      </c>
-      <c r="K18" t="s">
-        <v>18</v>
+      <c r="J18">
+        <v>200</v>
+      </c>
+      <c r="K18">
+        <v>15000</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H19" t="s">
         <v>63</v>
       </c>
       <c r="I19" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="J19" t="s">
         <v>18</v>
@@ -1574,22 +1625,22 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F20" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="G20" t="s">
         <v>18</v>
@@ -1609,28 +1660,28 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B21">
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F21" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H21" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="I21" t="s">
         <v>18</v>
@@ -1644,31 +1695,31 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G22" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="H22" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I22" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="J22" t="s">
         <v>18</v>
@@ -1679,22 +1730,22 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F23" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G23" t="s">
         <v>18</v>
@@ -1714,92 +1765,92 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F24" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G24" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="H24" t="s">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="I24" t="s">
-        <v>42</v>
-      </c>
-      <c r="J24" t="s">
-        <v>18</v>
-      </c>
-      <c r="K24" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="J24">
+        <v>200</v>
+      </c>
+      <c r="K24">
+        <v>15000</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F25" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G25" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H25" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="I25" t="s">
-        <v>18</v>
-      </c>
-      <c r="J25">
-        <v>200</v>
-      </c>
-      <c r="K25">
-        <v>15000</v>
+        <v>34</v>
+      </c>
+      <c r="J25" t="s">
+        <v>18</v>
+      </c>
+      <c r="K25" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D26" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G26" t="s">
         <v>18</v>
@@ -1810,46 +1861,361 @@
       <c r="I26" t="s">
         <v>18</v>
       </c>
-      <c r="J26" t="s">
-        <v>18</v>
-      </c>
-      <c r="K26" t="s">
-        <v>18</v>
+      <c r="J26">
+        <v>200</v>
+      </c>
+      <c r="K26">
+        <v>15000</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27" t="s">
         <v>74</v>
       </c>
-      <c r="B27">
+      <c r="I27" t="s">
+        <v>43</v>
+      </c>
+      <c r="J27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" t="s">
+        <v>36</v>
+      </c>
+      <c r="F28" t="s">
+        <v>45</v>
+      </c>
+      <c r="G28" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28">
+        <v>200</v>
+      </c>
+      <c r="K28">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29">
+        <v>5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29" t="s">
+        <v>30</v>
+      </c>
+      <c r="F29" t="s">
+        <v>31</v>
+      </c>
+      <c r="G29" t="s">
+        <v>48</v>
+      </c>
+      <c r="H29" t="s">
+        <v>76</v>
+      </c>
+      <c r="I29" t="s">
+        <v>50</v>
+      </c>
+      <c r="J29" t="s">
+        <v>18</v>
+      </c>
+      <c r="K29" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30">
+        <v>6</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30">
+        <v>200</v>
+      </c>
+      <c r="K30">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31">
+        <v>7</v>
+      </c>
+      <c r="C31" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31" t="s">
+        <v>36</v>
+      </c>
+      <c r="F31" t="s">
+        <v>40</v>
+      </c>
+      <c r="G31" t="s">
+        <v>18</v>
+      </c>
+      <c r="H31" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31">
+        <v>200</v>
+      </c>
+      <c r="K31">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" t="s">
+        <v>36</v>
+      </c>
+      <c r="F32" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32">
+        <v>200</v>
+      </c>
+      <c r="K32">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33">
         <v>2</v>
       </c>
-      <c r="C27" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C33" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" t="s">
         <v>13</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E33" t="s">
         <v>14</v>
       </c>
-      <c r="F27" t="s">
-        <v>78</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="F33" t="s">
+        <v>81</v>
+      </c>
+      <c r="G33" t="s">
         <v>16</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H33" t="s">
+        <v>82</v>
+      </c>
+      <c r="I33" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>83</v>
+      </c>
+      <c r="D34" t="s">
+        <v>84</v>
+      </c>
+      <c r="E34" t="s">
+        <v>30</v>
+      </c>
+      <c r="F34" t="s">
+        <v>85</v>
+      </c>
+      <c r="G34" t="s">
+        <v>32</v>
+      </c>
+      <c r="H34" t="s">
+        <v>86</v>
+      </c>
+      <c r="I34" t="s">
+        <v>87</v>
+      </c>
+      <c r="J34" t="s">
+        <v>18</v>
+      </c>
+      <c r="K34" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" t="s">
+        <v>36</v>
+      </c>
+      <c r="F35" t="s">
+        <v>89</v>
+      </c>
+      <c r="G35" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35">
+        <v>200</v>
+      </c>
+      <c r="K35">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" t="s">
         <v>79</v>
       </c>
-      <c r="I27" t="s">
-        <v>18</v>
-      </c>
-      <c r="J27" t="s">
-        <v>18</v>
-      </c>
-      <c r="K27" t="s">
-        <v>18</v>
+      <c r="E36" t="s">
+        <v>36</v>
+      </c>
+      <c r="F36" t="s">
+        <v>40</v>
+      </c>
+      <c r="G36" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36">
+        <v>200</v>
+      </c>
+      <c r="K36">
+        <v>15000</v>
       </c>
     </row>
   </sheetData>
@@ -1860,7 +2226,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1868,10 +2234,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -1891,10 +2257,10 @@
         <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1902,16 +2268,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3">
         <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1919,16 +2285,16 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>200</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E4" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1936,16 +2302,16 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5">
         <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1953,16 +2319,16 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6">
         <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1970,16 +2336,16 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7">
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1987,67 +2353,67 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8">
         <v>200</v>
       </c>
       <c r="D8" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="C9">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C10">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C11">
         <v>200</v>
       </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2055,16 +2421,16 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="C12">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D12" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2072,16 +2438,16 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C13">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E13" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2089,118 +2455,118 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C14">
         <v>200</v>
       </c>
       <c r="D14" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="C15">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D15" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C16">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E16" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C17">
         <v>200</v>
       </c>
       <c r="D17" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E17" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C18">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C19">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C20">
         <v>200</v>
       </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2208,55 +2574,55 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C21">
         <v>200</v>
       </c>
       <c r="D21" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="C22">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C23">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
         <v>65</v>
@@ -2265,146 +2631,299 @@
         <v>200</v>
       </c>
       <c r="D24" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s">
         <v>67</v>
       </c>
       <c r="C25">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D25" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="C26">
         <v>200</v>
       </c>
       <c r="D26" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E26" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C27">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D27" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="C28">
         <v>200</v>
       </c>
       <c r="D28" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C29">
         <v>202</v>
       </c>
       <c r="D29" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C30">
         <v>200</v>
       </c>
       <c r="D30" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E30" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C31">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D31" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32">
+        <v>200</v>
+      </c>
+      <c r="D32" t="s">
+        <v>93</v>
+      </c>
+      <c r="E32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33">
+        <v>202</v>
+      </c>
+      <c r="D33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34">
+        <v>200</v>
+      </c>
+      <c r="D34" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35">
+        <v>200</v>
+      </c>
+      <c r="D35" t="s">
+        <v>93</v>
+      </c>
+      <c r="E35" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>77</v>
       </c>
-      <c r="C32">
+      <c r="B36" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36">
+        <v>200</v>
+      </c>
+      <c r="D36" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" t="s">
+        <v>80</v>
+      </c>
+      <c r="C37">
         <v>403</v>
       </c>
-      <c r="D32" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" t="s">
-        <v>97</v>
+      <c r="D37" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38">
+        <v>200</v>
+      </c>
+      <c r="D38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39">
+        <v>202</v>
+      </c>
+      <c r="D39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>88</v>
+      </c>
+      <c r="C40">
+        <v>200</v>
+      </c>
+      <c r="D40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
+        <v>90</v>
+      </c>
+      <c r="C41">
+        <v>200</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V02-3 e V02-4: limite de posição e venda a descoberto com limite de exposição
Limite de 50.000 por conta e ativo (robô 200.000) por UPDATE condicional
em custodia_risco.compra_aberta (ADR-020). Venda além da custódia reserva
garantia em caixa e exposição até R$ 200.000,00 por conta, liberadas no
encerramento e na recompra D+2 (ADR-021, proposta pendente de confirmação).
Motivos LIMITE_POSICAO_EXCEDIDO e EXPOSICAO_VENDIDA_EXCEDIDA no FO, OpenAPI
e boleta; PlanoDeContas.d2 único construtor do lançamento D+2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/risco.xlsx
+++ b/frontend/runner/exemplos/risco.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="120">
   <si>
     <t>cenario</t>
   </si>
@@ -75,7 +75,7 @@
     <t>ReservaCustodia</t>
   </si>
   <si>
-    <t>{"saldo":"150.00","custodia":{"GAMA3":5}}</t>
+    <t>{"saldo":"400.00","custodia":{"GAMA3":5}}</t>
   </si>
   <si>
     <t>MarketTeto</t>
@@ -183,22 +183,25 @@
     <t>{"ticker":"GAMA3","lado":"VENDA","tipo":"LIMIT","validade":"DIA","quantidade":6,"precoLimite":"30.00"}</t>
   </si>
   <si>
-    <t>ExcedenteRejeitada</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>{"ticker":"GAMA3","lado":"VENDA","tipo":"LIMIT","validade":"DIA","quantidade":5,"precoLimite":"30.00"}</t>
-  </si>
-  <si>
-    <t>TotalReservada</t>
-  </si>
-  <si>
-    <t>CustodiaReservada</t>
-  </si>
-  <si>
-    <t>{"ticker":"GAMA3","lado":"COMPRA","tipo":"LIMIT","validade":"IOC","quantidade":5,"precoLimite":"30.00"}</t>
+    <t>ExcedenteReservada</t>
+  </si>
+  <si>
+    <t>CustodiaEGarantia</t>
+  </si>
+  <si>
+    <t>SemGarantia</t>
+  </si>
+  <si>
+    <t>{"ticker":"GAMA3","lado":"VENDA","tipo":"LIMIT","validade":"DIA","quantidade":12,"precoLimite":"30.00"}</t>
+  </si>
+  <si>
+    <t>SemGarantiaRejeitada</t>
+  </si>
+  <si>
+    <t>{"ticker":"GAMA3","lado":"COMPRA","tipo":"LIMIT","validade":"IOC","quantidade":6,"precoLimite":"30.00"}</t>
+  </si>
+  <si>
+    <t>VendidoAteOD2</t>
   </si>
   <si>
     <t>Insuficiente</t>
@@ -228,22 +231,34 @@
     <t>Acima</t>
   </si>
   <si>
-    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100001,"precoLimite":"10.00"}</t>
+    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"DIA","quantidade":100001,"precoLimite":"11.00"}</t>
   </si>
   <si>
     <t>AcimaRejeitada</t>
   </si>
   <si>
+    <t>LimitePosicao</t>
+  </si>
+  <si>
+    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":1,"precoLimite":"10.00"}</t>
+  </si>
+  <si>
+    <t>LimitePosicaoRejeitada</t>
+  </si>
+  <si>
     <t>NoLimite</t>
   </si>
   <si>
-    <t>{"ticker":"ALFA3","lado":"COMPRA","tipo":"LIMIT","validade":"DIA","quantidade":100000,"precoLimite":"10.00"}</t>
-  </si>
-  <si>
-    <t>NoLimiteReservada</t>
-  </si>
-  <si>
-    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"IOC","quantidade":100000,"precoLimite":"10.00"}</t>
+    <t>{"ticker":"ALFA3","lado":"VENDA","tipo":"LIMIT","validade":"IOC","quantidade":100000,"precoLimite":"11.00"}</t>
+  </si>
+  <si>
+    <t>{"id3":"/id"}</t>
+  </si>
+  <si>
+    <t>NoLimiteEncerrada</t>
+  </si>
+  <si>
+    <t>/api/v1/ordens/${id3}</t>
   </si>
   <si>
     <t>Isolamento</t>
@@ -318,13 +333,10 @@
     <t>{"/saldoTotal":"30.00","/saldoReservado":"0.00"}</t>
   </si>
   <si>
-    <t>{"/estado":"REJEITADA","/motivoRejeicao":"CUSTODIA_INSUFICIENTE"}</t>
-  </si>
-  <si>
-    <t>{"/custodias/3/ticker":"GAMA3","/custodias/3/disponivel":0,"/custodias/3/reservado":5}</t>
-  </si>
-  <si>
-    <t>{"/saldoTotal":"0.00","/saldoReservado":"0.00","/custodias/3/reservado":0}</t>
+    <t>{"/saldoDisponivel":"367.00","/saldoReservado":"33.00","/exposicaoVendida":"30.00","/custodias/3/ticker":"GAMA3","/custodias/3/disponivel":0,"/custodias/3/reservado":5,"/custodias/3/descobertoReservado":1}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"220.00","/saldoReservado":"33.00","/exposicaoVendida":"30.00","/custodias/3/total":0,"/custodias/3/reservado":0,"/custodias/3/descobertoReservado":0,"/custodias/3/descobertoExecutado":1}</t>
   </si>
   <si>
     <t>{"/saldoDisponivel":"220.00"}</t>
@@ -339,7 +351,10 @@
     <t>{"/estado":"REJEITADA","/motivoRejeicao":"QUANTIDADE_MAXIMA_EXCEDIDA"}</t>
   </si>
   <si>
-    <t>{"/saldoTotal":"1000000.00","/saldoReservado":"0.00"}</t>
+    <t>{"/estado":"REJEITADA","/motivoRejeicao":"LIMITE_POSICAO_EXCEDIDO"}</t>
+  </si>
+  <si>
+    <t>{"/saldoTotal":"2000000.00","/saldoReservado":"0.00","/custodias/0/ticker":"ALFA3","/custodias/0/reservado":0}</t>
   </si>
   <si>
     <t>{"/conta":"CONTA-003"}</t>
@@ -1389,28 +1404,28 @@
         <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G13" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="H13" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="I13" t="s">
-        <v>43</v>
-      </c>
-      <c r="J13" t="s">
-        <v>18</v>
-      </c>
-      <c r="K13" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="J13">
+        <v>200</v>
+      </c>
+      <c r="K13">
+        <v>15000</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1421,31 +1436,31 @@
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="G14" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
-        <v>18</v>
-      </c>
-      <c r="J14">
-        <v>200</v>
-      </c>
-      <c r="K14">
-        <v>15000</v>
+        <v>43</v>
+      </c>
+      <c r="J14" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1459,13 +1474,13 @@
         <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
         <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G15" t="s">
         <v>18</v>
@@ -1561,7 +1576,7 @@
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
         <v>39</v>
@@ -1596,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
         <v>29</v>
@@ -1611,7 +1626,7 @@
         <v>32</v>
       </c>
       <c r="H19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I19" t="s">
         <v>34</v>
@@ -1631,7 +1646,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" t="s">
         <v>29</v>
@@ -1666,7 +1681,7 @@
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
         <v>13</v>
@@ -1681,7 +1696,7 @@
         <v>16</v>
       </c>
       <c r="H21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I21" t="s">
         <v>18</v>
@@ -1701,7 +1716,7 @@
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D22" t="s">
         <v>29</v>
@@ -1716,7 +1731,7 @@
         <v>42</v>
       </c>
       <c r="H22" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I22" t="s">
         <v>43</v>
@@ -1736,7 +1751,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
@@ -1771,7 +1786,7 @@
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D24" t="s">
         <v>39</v>
@@ -1806,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
         <v>29</v>
@@ -1821,7 +1836,7 @@
         <v>32</v>
       </c>
       <c r="H25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I25" t="s">
         <v>34</v>
@@ -1841,7 +1856,7 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D26" t="s">
         <v>29</v>
@@ -1876,7 +1891,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1891,7 +1906,7 @@
         <v>42</v>
       </c>
       <c r="H27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I27" t="s">
         <v>43</v>
@@ -1911,7 +1926,7 @@
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D28" t="s">
         <v>29</v>
@@ -1946,7 +1961,7 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
         <v>29</v>
@@ -1961,10 +1976,10 @@
         <v>48</v>
       </c>
       <c r="H29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I29" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="J29" t="s">
         <v>18</v>
@@ -1981,7 +1996,7 @@
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="D30" t="s">
         <v>29</v>
@@ -1990,7 +2005,7 @@
         <v>36</v>
       </c>
       <c r="F30" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="G30" t="s">
         <v>18</v>
@@ -2045,16 +2060,16 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D32" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E32" t="s">
         <v>36</v>
@@ -2080,13 +2095,13 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D33" t="s">
         <v>13</v>
@@ -2095,13 +2110,13 @@
         <v>14</v>
       </c>
       <c r="F33" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G33" t="s">
         <v>16</v>
       </c>
       <c r="H33" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="I33" t="s">
         <v>18</v>
@@ -2121,25 +2136,25 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D34" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E34" t="s">
         <v>30</v>
       </c>
       <c r="F34" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G34" t="s">
         <v>32</v>
       </c>
       <c r="H34" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="I34" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J34" t="s">
         <v>18</v>
@@ -2156,16 +2171,16 @@
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D35" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E35" t="s">
         <v>36</v>
       </c>
       <c r="F35" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G35" t="s">
         <v>18</v>
@@ -2191,10 +2206,10 @@
         <v>3</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D36" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E36" t="s">
         <v>36</v>
@@ -2234,10 +2249,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -2257,10 +2272,10 @@
         <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2274,10 +2289,10 @@
         <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2291,10 +2306,10 @@
         <v>200</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2308,10 +2323,10 @@
         <v>200</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2325,10 +2340,10 @@
         <v>202</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2342,10 +2357,10 @@
         <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2359,10 +2374,10 @@
         <v>200</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2376,10 +2391,10 @@
         <v>202</v>
       </c>
       <c r="D9" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2393,10 +2408,10 @@
         <v>200</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E10" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2410,10 +2425,10 @@
         <v>200</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2427,10 +2442,10 @@
         <v>200</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E12" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2444,10 +2459,10 @@
         <v>202</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E13" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2461,7 +2476,7 @@
         <v>200</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E14" t="s">
         <v>101</v>
@@ -2475,13 +2490,13 @@
         <v>57</v>
       </c>
       <c r="C15">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E15" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -2489,16 +2504,16 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C16">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2512,10 +2527,10 @@
         <v>200</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2529,10 +2544,10 @@
         <v>202</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -2546,10 +2561,10 @@
         <v>200</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E19" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -2557,16 +2572,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="C20">
         <v>200</v>
       </c>
       <c r="D20" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E20" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2580,10 +2595,10 @@
         <v>200</v>
       </c>
       <c r="D21" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2591,16 +2606,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22">
         <v>202</v>
       </c>
       <c r="D22" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -2608,16 +2623,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23">
         <v>200</v>
       </c>
       <c r="D23" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -2625,16 +2640,16 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24">
         <v>200</v>
       </c>
       <c r="D24" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E24" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -2642,16 +2657,16 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C25">
         <v>202</v>
       </c>
       <c r="D25" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E25" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -2659,16 +2674,16 @@
         <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26">
         <v>200</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E26" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -2676,16 +2691,16 @@
         <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27">
         <v>200</v>
       </c>
       <c r="D27" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E27" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -2699,10 +2714,10 @@
         <v>200</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E28" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -2710,16 +2725,16 @@
         <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C29">
         <v>202</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E29" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -2727,16 +2742,16 @@
         <v>23</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C30">
         <v>200</v>
       </c>
       <c r="D30" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E30" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -2744,16 +2759,16 @@
         <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C31">
         <v>202</v>
       </c>
       <c r="D31" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E31" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -2761,16 +2776,16 @@
         <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32">
         <v>200</v>
       </c>
       <c r="D32" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -2778,16 +2793,16 @@
         <v>23</v>
       </c>
       <c r="B33" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="C33">
         <v>202</v>
       </c>
       <c r="D33" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E33" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -2795,16 +2810,16 @@
         <v>23</v>
       </c>
       <c r="B34" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="C34">
         <v>200</v>
       </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E34" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -2818,44 +2833,44 @@
         <v>200</v>
       </c>
       <c r="D35" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E35" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B36" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C36">
         <v>200</v>
       </c>
       <c r="D36" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E36" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C37">
         <v>403</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E37" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -2869,10 +2884,10 @@
         <v>200</v>
       </c>
       <c r="D38" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E38" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -2880,16 +2895,16 @@
         <v>25</v>
       </c>
       <c r="B39" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C39">
         <v>202</v>
       </c>
       <c r="D39" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E39" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -2897,16 +2912,16 @@
         <v>25</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C40">
         <v>200</v>
       </c>
       <c r="D40" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E40" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2914,16 +2929,16 @@
         <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C41">
         <v>200</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E41" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>